<commit_message>
Align Correct Score features with backtest and fix staleness and name normalizations
</commit_message>
<xml_diff>
--- a/coleta_lay0x2_aovivo.xlsx
+++ b/coleta_lay0x2_aovivo.xlsx
@@ -580,11 +580,15 @@
           <t>RF</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>98.3</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>20</v>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>98.3</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="I2" s="4" t="inlineStr"/>
       <c r="J2" s="4" t="inlineStr"/>

</xml_diff>